<commit_message>
PID controller tuned -> max 760 Nm Tq limit stll there
</commit_message>
<xml_diff>
--- a/documentation/labcar_integration_planning.xlsx
+++ b/documentation/labcar_integration_planning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work_local_TimBein\GVCU_HIL_repo\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DBBA342-9585-4A39-A23F-377CD2A45302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17E9BEAB-C863-4166-AAB5-86B4594E00B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{D929C58B-B70F-4223-A9B1-326C665B473E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{D929C58B-B70F-4223-A9B1-326C665B473E}"/>
   </bookViews>
   <sheets>
     <sheet name="CAN" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="70">
   <si>
     <t>GVCU BUS</t>
   </si>
@@ -419,7 +419,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -427,14 +427,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -503,13 +502,12 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -523,9 +521,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -539,7 +534,207 @@
   </cellStyles>
   <dxfs count="14">
     <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -692,207 +887,7 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -911,28 +906,28 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37185F8D-FEE7-4090-A4CD-3A74C40F5CD7}" name="Table1" displayName="Table1" ref="B2:H36" totalsRowShown="0">
   <autoFilter ref="B2:H36" xr:uid="{37185F8D-FEE7-4090-A4CD-3A74C40F5CD7}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D163736F-60C4-4242-B51E-116DE7F34AEA}" name="GVCU BUS" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{82988792-2CCC-40E2-AEF1-D28A21188844}" name="Tx VT System" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{C1C73E01-54E7-45A0-83E3-21641927E824}" name="Rx VT System" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{6FCB88D9-8D84-48DA-A02C-88F832ACCEF2}" name="Relevant CAN-Signal" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{C1C0A43F-0491-4D99-96C8-A12AF5B141B6}" name="Real Car origin" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{544452DA-E2B3-4438-888A-8FC2321F47E4}" name="Labcar options" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{3978658B-E62F-491C-B9D8-0D1407B02827}" name="Checked importance" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{D163736F-60C4-4242-B51E-116DE7F34AEA}" name="GVCU BUS" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{82988792-2CCC-40E2-AEF1-D28A21188844}" name="Tx VT System" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{C1C73E01-54E7-45A0-83E3-21641927E824}" name="Rx VT System" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{6FCB88D9-8D84-48DA-A02C-88F832ACCEF2}" name="Relevant CAN-Signal" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{C1C0A43F-0491-4D99-96C8-A12AF5B141B6}" name="Real Car origin" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{544452DA-E2B3-4438-888A-8FC2321F47E4}" name="Labcar options" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{3978658B-E62F-491C-B9D8-0D1407B02827}" name="Checked importance" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D7A9D742-81F4-4A25-8D90-441E5A2563D1}" name="Table15" displayName="Table15" ref="B2:G15" totalsRowShown="0" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D7A9D742-81F4-4A25-8D90-441E5A2563D1}" name="Table15" displayName="Table15" ref="B2:G15" totalsRowShown="0" dataDxfId="13">
   <autoFilter ref="B2:G15" xr:uid="{D7A9D742-81F4-4A25-8D90-441E5A2563D1}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{1BF40364-91FB-4842-9839-531ED49CA30C}" name="VT System" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{2290D721-548C-444B-A533-111B16D87FDC}" name="Purpose" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{F159257B-D8BB-48D3-A82B-E2E7D2852BAA}" name="Column1" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{75CB03C2-8E07-44B9-8C90-824A464391AE}" name="Real Car origin" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{59D8879F-5AFB-48E3-BC9B-96834185A3D1}" name="Labcar options" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{7F11F261-C389-4CE6-88A9-9CFD1B13FD78}" name="Checked importance" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{1BF40364-91FB-4842-9839-531ED49CA30C}" name="VT System" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{2290D721-548C-444B-A533-111B16D87FDC}" name="Purpose" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{F159257B-D8BB-48D3-A82B-E2E7D2852BAA}" name="Column1" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{75CB03C2-8E07-44B9-8C90-824A464391AE}" name="Real Car origin" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{59D8879F-5AFB-48E3-BC9B-96834185A3D1}" name="Labcar options" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{7F11F261-C389-4CE6-88A9-9CFD1B13FD78}" name="Checked importance" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1299,9 +1294,9 @@
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="34"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="33"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" s="5"/>
@@ -1310,9 +1305,11 @@
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" s="5"/>
@@ -1321,9 +1318,9 @@
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" s="5"/>
@@ -1332,9 +1329,9 @@
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="5"/>
@@ -1343,9 +1340,9 @@
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" s="5"/>
@@ -1354,9 +1351,9 @@
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="5"/>
@@ -1365,9 +1362,9 @@
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" s="5"/>
@@ -1375,12 +1372,12 @@
         <v>18</v>
       </c>
       <c r="D10" s="7"/>
-      <c r="E10" s="49" t="s">
+      <c r="E10" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="5"/>
@@ -1389,9 +1386,9 @@
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" spans="2:8" ht="29" x14ac:dyDescent="0.35">
       <c r="B12" s="5"/>
@@ -1399,297 +1396,297 @@
         <v>16</v>
       </c>
       <c r="D12" s="7"/>
-      <c r="E12" s="50" t="s">
+      <c r="E12" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8" t="s">
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
     </row>
     <row r="14" spans="2:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="B14" s="8"/>
-      <c r="C14" s="8" t="s">
+      <c r="B14" s="5"/>
+      <c r="C14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="56" t="s">
+      <c r="D14" s="5"/>
+      <c r="E14" s="54" t="s">
         <v>45</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8" t="s">
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="B15" s="59"/>
-      <c r="C15" s="59" t="s">
+      <c r="B15" s="57"/>
+      <c r="C15" s="57" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="59"/>
-      <c r="E15" s="60" t="s">
+      <c r="D15" s="57"/>
+      <c r="E15" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="F15" s="59"/>
-      <c r="G15" s="59"/>
-      <c r="H15" s="8"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="5"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B16" s="59"/>
-      <c r="C16" s="59"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="59"/>
-      <c r="H16" s="8"/>
+      <c r="B16" s="57"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="58"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="5"/>
     </row>
     <row r="17" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="51"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="55"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="29"/>
+      <c r="B17" s="50"/>
+      <c r="C17" s="51"/>
+      <c r="D17" s="52"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="50"/>
+      <c r="G17" s="50"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="35" t="s">
+      <c r="B18" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="36"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="44"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="43"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="32"/>
-      <c r="E19" s="33" t="s">
+      <c r="D19" s="31"/>
+      <c r="E19" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="8"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="5"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="57"/>
-      <c r="C20" s="9" t="s">
+      <c r="B20" s="55"/>
+      <c r="C20" s="8" t="s">
         <v>22</v>
       </c>
       <c r="D20" s="7"/>
-      <c r="E20" s="33" t="s">
+      <c r="E20" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
       <c r="J20" s="5"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B21" s="57"/>
-      <c r="C21" s="13" t="s">
+      <c r="B21" s="55"/>
+      <c r="C21" s="12" t="s">
         <v>49</v>
       </c>
       <c r="D21" s="7"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
     </row>
     <row r="22" spans="2:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="B22" s="13"/>
-      <c r="C22" s="16" t="s">
+      <c r="B22" s="12"/>
+      <c r="C22" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D22" s="17"/>
-      <c r="E22" s="58" t="s">
+      <c r="D22" s="16"/>
+      <c r="E22" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8" t="s">
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="23" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="25"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="27" t="s">
+      <c r="B23" s="24"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E23" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="29"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="28"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="12"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="11"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B25" s="10"/>
-      <c r="C25" s="14" t="s">
+      <c r="B25" s="9"/>
+      <c r="C25" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B26" s="10"/>
-      <c r="C26" s="14" t="s">
+      <c r="B26" s="9"/>
+      <c r="C26" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B27" s="10"/>
-      <c r="C27" s="14" t="s">
+      <c r="B27" s="9"/>
+      <c r="C27" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B28" s="10"/>
-      <c r="C28" s="14" t="s">
+      <c r="B28" s="9"/>
+      <c r="C28" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B29" s="10"/>
-      <c r="C29" s="14" t="s">
+      <c r="B29" s="9"/>
+      <c r="C29" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B30" s="10"/>
-      <c r="C30" s="14" t="s">
+      <c r="B30" s="9"/>
+      <c r="C30" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B31" s="10"/>
-      <c r="C31" s="14" t="s">
+      <c r="B31" s="9"/>
+      <c r="C31" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B32" s="10"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="15" t="s">
+      <c r="B32" s="9"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="15"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
     </row>
     <row r="33" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B33" s="41"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="43" t="s">
+      <c r="B33" s="40"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="E33" s="43"/>
-      <c r="F33" s="44"/>
-      <c r="G33" s="44"/>
-      <c r="H33" s="44"/>
+      <c r="E33" s="42"/>
+      <c r="F33" s="43"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="43"/>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="19" t="s">
         <v>8</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="18"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="17"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B35" s="19"/>
+      <c r="B35" s="18"/>
       <c r="C35" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
     </row>
     <row r="36" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B36" s="45"/>
-      <c r="C36" s="46" t="s">
+      <c r="B36" s="44"/>
+      <c r="C36" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="47"/>
-      <c r="E36" s="47"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="48"/>
-      <c r="H36" s="29"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="47"/>
+      <c r="G36" s="47"/>
+      <c r="H36" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1734,168 +1731,168 @@
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B3" s="62" t="s">
+      <c r="B3" s="60" t="s">
         <v>55</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>59</v>
       </c>
       <c r="D3" s="7"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="64" t="s">
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="61" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="60" t="s">
         <v>56</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>59</v>
       </c>
       <c r="D4" s="7"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63" t="s">
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B5" s="62"/>
+      <c r="B5" s="60"/>
       <c r="C5" s="6"/>
       <c r="D5" s="7"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="60" t="s">
         <v>60</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="64" t="s">
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="61" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B7" s="62" t="s">
+      <c r="B7" s="60" t="s">
         <v>61</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D7" s="7"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63" t="s">
+      <c r="E7" s="60"/>
+      <c r="F7" s="60"/>
+      <c r="G7" s="60" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="60" t="s">
         <v>62</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D8" s="7"/>
-      <c r="E8" s="63"/>
-      <c r="F8" s="63"/>
-      <c r="G8" s="64" t="s">
+      <c r="E8" s="60"/>
+      <c r="F8" s="60"/>
+      <c r="G8" s="61" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B9" s="62" t="s">
+      <c r="B9" s="60" t="s">
         <v>63</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D9" s="7"/>
-      <c r="E9" s="63"/>
-      <c r="F9" s="63"/>
-      <c r="G9" s="63" t="s">
+      <c r="E9" s="60"/>
+      <c r="F9" s="60"/>
+      <c r="G9" s="60" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B10" s="62"/>
+      <c r="B10" s="60"/>
       <c r="C10" s="6"/>
       <c r="D10" s="7"/>
-      <c r="E10" s="63"/>
-      <c r="F10" s="63"/>
-      <c r="G10" s="63"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
     </row>
     <row r="11" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="62" t="s">
+      <c r="B11" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="59" t="s">
         <v>69</v>
       </c>
       <c r="D11" s="7"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
-      <c r="G11" s="64" t="s">
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="61" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="62" t="s">
+      <c r="B12" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="C12" s="61" t="s">
+      <c r="C12" s="59" t="s">
         <v>69</v>
       </c>
       <c r="D12" s="7"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
-      <c r="G12" s="63" t="s">
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="60" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B13" s="62" t="s">
+      <c r="B13" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="61" t="s">
+      <c r="C13" s="59" t="s">
         <v>69</v>
       </c>
       <c r="D13" s="7"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
-      <c r="G13" s="64" t="s">
+      <c r="E13" s="60"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="61" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B14" s="62" t="s">
+      <c r="B14" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="C14" s="61" t="s">
+      <c r="C14" s="59" t="s">
         <v>69</v>
       </c>
       <c r="D14" s="7"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
-      <c r="G14" s="63" t="s">
+      <c r="E14" s="60"/>
+      <c r="F14" s="60"/>
+      <c r="G14" s="60" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B15" s="62"/>
+      <c r="B15" s="60"/>
       <c r="C15" s="6"/>
       <c r="D15" s="7"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
-      <c r="G15" s="63"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="60"/>
+      <c r="G15" s="60"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>